<commit_message>
Attempting to Combine code.. Added files
</commit_message>
<xml_diff>
--- a/Code/Matlab/Analysis/Dynamic_Simulation/Muscle_Data.xlsx
+++ b/Code/Matlab/Analysis/Dynamic_Simulation/Muscle_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnstr\Documents\GitHub\Quad\Code\Matlab\Analysis\Dynamic_Simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FED586D6-46CC-4AC9-94DC-252C1ED0B8DD}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3801DF-7138-4DEB-A103-F97A046E4506}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{999E1B3B-F109-4E43-8C1D-5C150D6805EA}"/>
+    <workbookView xWindow="10755" yWindow="2775" windowWidth="12825" windowHeight="12165" xr2:uid="{999E1B3B-F109-4E43-8C1D-5C150D6805EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
   <si>
     <t>Muscle Name</t>
   </si>
@@ -130,6 +130,12 @@
   </si>
   <si>
     <t>Joint_3</t>
+  </si>
+  <si>
+    <t>Ma Hip Add</t>
+  </si>
+  <si>
+    <t>Ma Hip Abd</t>
   </si>
 </sst>
 </file>
@@ -485,7 +491,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C8D057-9905-4E8D-B3F8-C044FC33D5F2}">
-  <dimension ref="A1:P11"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
@@ -1030,6 +1036,98 @@
         <v>0.39553468623009591</v>
       </c>
     </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="C12" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12">
+        <v>3.5209999999999998E-2</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0.22434999999999999</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>3.4009999999999999E-2</v>
+      </c>
+      <c r="J12">
+        <v>0.24123</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>3.4009999999999999E-2</v>
+      </c>
+      <c r="M12">
+        <v>1</v>
+      </c>
+      <c r="N12">
+        <v>2</v>
+      </c>
+      <c r="O12">
+        <v>2</v>
+      </c>
+      <c r="P12">
+        <f>SQRT((G13-D13)^2+(H13+E13)^2+(I13+F13)^2)+SQRT((J13-G13)^2+(K13+H13)^2+(L13+I13)^2)</f>
+        <v>0.38346906734938946</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>33</v>
+      </c>
+      <c r="C13" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13">
+        <v>3.5209999999999998E-2</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>9.6509999999999999E-2</v>
+      </c>
+      <c r="G13">
+        <v>0.22434999999999999</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>6.6390000000000005E-2</v>
+      </c>
+      <c r="J13">
+        <v>0.24123</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>6.6390000000000005E-2</v>
+      </c>
+      <c r="M13">
+        <v>1</v>
+      </c>
+      <c r="N13">
+        <v>2</v>
+      </c>
+      <c r="O13">
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="D1:F1"/>
@@ -1037,10 +1135,10 @@
     <mergeCell ref="J1:L1"/>
   </mergeCells>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B6 B7:B11" xr:uid="{A9258D5C-1BC9-44B6-9026-07535BA2D0A9}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B3:B11" xr:uid="{A9258D5C-1BC9-44B6-9026-07535BA2D0A9}">
       <formula1>"Ext, Flx"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:C6 C7:C11" xr:uid="{BFD3125F-7AA0-4ADB-A941-68410798869E}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C3:C11" xr:uid="{BFD3125F-7AA0-4ADB-A941-68410798869E}">
       <formula1>"Mono, Bi"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Combined simulation works without abduction/adduction
</commit_message>
<xml_diff>
--- a/Code/Matlab/Analysis/Dynamic_Simulation/Muscle_Data.xlsx
+++ b/Code/Matlab/Analysis/Dynamic_Simulation/Muscle_Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnstr\Documents\GitHub\Quad\Code\Matlab\Analysis\Dynamic_Simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C3801DF-7138-4DEB-A103-F97A046E4506}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3FE317-0FDB-4386-810F-D8980CC1A80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10755" yWindow="2775" windowWidth="12825" windowHeight="12165" xr2:uid="{999E1B3B-F109-4E43-8C1D-5C150D6805EA}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{999E1B3B-F109-4E43-8C1D-5C150D6805EA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
   <si>
     <t>Muscle Name</t>
   </si>
@@ -82,9 +82,6 @@
   </si>
   <si>
     <t>Bi</t>
-  </si>
-  <si>
-    <t>Resting Length (m)</t>
   </si>
   <si>
     <t>First Point (m from origin)</t>
@@ -173,10 +170,10 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -491,7 +488,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C8D057-9905-4E8D-B3F8-C044FC33D5F2}">
-  <dimension ref="A1:P13"/>
+  <dimension ref="A1:O13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
@@ -509,25 +506,25 @@
     <col min="16" max="16" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
-      <c r="D1" s="1" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="D1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
-      <c r="O1" s="2"/>
-    </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="O1" s="1"/>
+    </row>
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -538,46 +535,43 @@
         <v>2</v>
       </c>
       <c r="D2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E2" t="s">
         <v>20</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>21</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>22</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>23</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>24</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>25</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>26</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>27</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>28</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>29</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>30</v>
       </c>
-      <c r="O2" t="s">
-        <v>31</v>
-      </c>
-      <c r="P2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -621,14 +615,10 @@
         <v>0</v>
       </c>
       <c r="O3">
-        <v>1</v>
-      </c>
-      <c r="P3">
-        <f>SQRT((G3-D3)^2+(H3+E3)^2+(I3+F3)^2)+SQRT((J3-G3)^2+(K3+H3)^2+(L3+I3)^2)</f>
-        <v>0.38881327881410749</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -672,14 +662,10 @@
         <v>0</v>
       </c>
       <c r="O4">
-        <v>1</v>
-      </c>
-      <c r="P4">
-        <f>SQRT((G4-D4)^2+(H4+E4)^2+(I4+F4)^2)+SQRT((J4-G4)^2+(K4+H4)^2+(L4+I4)^2)</f>
-        <v>0.40840306795131104</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -717,20 +703,16 @@
         <v>5.0201999999999997E-2</v>
       </c>
       <c r="M5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O5">
-        <v>2</v>
-      </c>
-      <c r="P5">
-        <f>SQRT((G5-D5)^2+(H5+E5)^2+(I5+F5)^2)+SQRT((J5-G5)^2+(K5+H5)^2+(L5+I5)^2)</f>
-        <v>0.4299493620499848</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -768,20 +750,16 @@
         <v>5.0201999999999997E-2</v>
       </c>
       <c r="M6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N6">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O6">
-        <v>2</v>
-      </c>
-      <c r="P6">
-        <f>SQRT((G6-D6)^2+(H6+E6)^2+(I6+F6)^2)+SQRT((J6-G6)^2+(K6+H6)^2+(L6+I6)^2)</f>
-        <v>0.43036655864928147</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -819,20 +797,16 @@
         <v>5.0265999999999998E-2</v>
       </c>
       <c r="M7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N7">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O7">
-        <v>3</v>
-      </c>
-      <c r="P7">
-        <f>SQRT((G7-D7)^2+(H7+E7)^2+(I7+F7)^2)+SQRT((J7-G7)^2+(K7+H7)^2+(L7+I7)^2)</f>
-        <v>0.33848182495506873</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -870,20 +844,16 @@
         <v>5.0265999999999998E-2</v>
       </c>
       <c r="M8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N8">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="O8">
-        <v>3</v>
-      </c>
-      <c r="P8">
-        <f>SQRT((G8-D8)^2+(H8+E8)^2+(I8+F8)^2)+SQRT((J8-G8)^2+(K8+H8)^2+(L8+I8)^2)</f>
-        <v>0.33503817437420658</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -924,17 +894,13 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O9">
-        <v>2</v>
-      </c>
-      <c r="P9">
-        <f>SQRT((G9-D9)^2+(H9+E9)^2+(I9+F9)^2)+SQRT((J9-G9)^2+(K9+H9)^2+(L9+I9)^2)</f>
-        <v>0.42571302901523833</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -975,17 +941,13 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10">
-        <v>2</v>
-      </c>
-      <c r="P10">
-        <f>SQRT((G10-D10)^2+(H10+E10)^2+(I10+F10)^2)+SQRT((J10-G10)^2+(K10+H10)^2+(L10+I10)^2)</f>
-        <v>0.34239955206255718</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -1023,22 +985,18 @@
         <v>5.0265999999999998E-2</v>
       </c>
       <c r="M11">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N11">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="O11">
-        <v>3</v>
-      </c>
-      <c r="P11">
-        <f>SQRT((G11-D11)^2+(H11+E11)^2+(I11+F11)^2)+SQRT((J11-G11)^2+(K11+H11)^2+(L11+I11)^2)</f>
-        <v>0.39553468623009591</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C12" t="s">
         <v>14</v>
@@ -1079,14 +1037,10 @@
       <c r="O12">
         <v>2</v>
       </c>
-      <c r="P12">
-        <f>SQRT((G13-D13)^2+(H13+E13)^2+(I13+F13)^2)+SQRT((J13-G13)^2+(K13+H13)^2+(L13+I13)^2)</f>
-        <v>0.38346906734938946</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C13" t="s">
         <v>14</v>

</xml_diff>

<commit_message>
updated muscle data to fit the final CAD Model
</commit_message>
<xml_diff>
--- a/Code/Matlab/Analysis/Dynamic_Simulation/Muscle_Data.xlsx
+++ b/Code/Matlab/Analysis/Dynamic_Simulation/Muscle_Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnstr\Documents\GitHub\Quad\Code\Matlab\Analysis\Dynamic_Simulation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3FE317-0FDB-4386-810F-D8980CC1A80F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40B712AC-464B-4C77-9654-36AB2F1D55CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{999E1B3B-F109-4E43-8C1D-5C150D6805EA}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="35">
   <si>
     <t>Muscle Name</t>
   </si>
@@ -133,12 +133,21 @@
   </si>
   <si>
     <t>Ma Hip Abd</t>
+  </si>
+  <si>
+    <t>initial length (m)</t>
+  </si>
+  <si>
+    <t>Initial length (in)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.000000"/>
+  </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -168,9 +177,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -488,43 +498,37 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{77C8D057-9905-4E8D-B3F8-C044FC33D5F2}">
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13" customWidth="1"/>
     <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="9" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="11" width="12.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="15" width="11.5703125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="16" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="D1" s="2" t="s">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+      <c r="D1" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2" t="s">
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2" t="s">
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
       <c r="O1" s="1"/>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -570,8 +574,14 @@
       <c r="O2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P2" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -581,44 +591,52 @@
       <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="2">
         <v>-0.38890000000000002</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="2">
         <v>1.11E-2</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="2">
         <v>-1.67E-2</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="2">
         <v>-8.4909999999999999E-2</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="2">
         <v>1.11E-2</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="2">
         <v>-1.67E-2</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="2">
         <v>-6.3499999999999997E-3</v>
       </c>
-      <c r="K3">
+      <c r="K3" s="2">
         <v>6.3499999999999997E-3</v>
       </c>
-      <c r="L3">
+      <c r="L3" s="2">
         <v>0</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="2">
         <v>0</v>
       </c>
-      <c r="N3">
+      <c r="N3" s="2">
         <v>0</v>
       </c>
-      <c r="O3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O3" s="2">
+        <v>2</v>
+      </c>
+      <c r="P3">
+        <f>SQRT((G3-D3)^2+(H3-E3)^2-(I3-F3)^2)</f>
+        <v>0.30399000000000004</v>
+      </c>
+      <c r="Q3">
+        <f>P3*39.37</f>
+        <v>11.968086300000001</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -628,44 +646,52 @@
       <c r="C4" t="s">
         <v>14</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="2">
         <v>-0.38890000000000002</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="2">
         <v>2.8575E-2</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="2">
         <v>-1.6669E-2</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="2">
         <v>-8.8900000000000007E-2</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="2">
         <v>2.8573999999999999E-2</v>
       </c>
-      <c r="I4">
+      <c r="I4" s="2">
         <v>-1.6669E-2</v>
       </c>
-      <c r="J4">
+      <c r="J4" s="2">
         <v>8.4060000000000003E-3</v>
       </c>
-      <c r="K4">
+      <c r="K4" s="2">
         <v>-6.3499999999999997E-3</v>
       </c>
-      <c r="L4">
+      <c r="L4" s="2">
         <v>0</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="2">
         <v>0</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="2">
         <v>0</v>
       </c>
-      <c r="O4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="O4" s="2">
+        <v>2</v>
+      </c>
+      <c r="P4">
+        <f t="shared" ref="P4:P13" si="0">SQRT((G4-D4)^2+(H4-E4)^2-(I4-F4)^2)</f>
+        <v>0.30000000000166671</v>
+      </c>
+      <c r="Q4">
+        <f t="shared" ref="Q4:Q13" si="1">P4*39.37</f>
+        <v>11.811000000065617</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -675,44 +701,52 @@
       <c r="C5" t="s">
         <v>14</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="2">
         <v>-4.8259999999999997E-2</v>
       </c>
-      <c r="E5">
-        <v>-2.1590000000000002E-2</v>
-      </c>
-      <c r="F5">
+      <c r="E5" s="2">
+        <v>-2.0409E-2</v>
+      </c>
+      <c r="F5" s="2">
         <v>5.0075000000000001E-2</v>
       </c>
-      <c r="G5">
-        <v>0.26194499999999998</v>
-      </c>
-      <c r="H5">
-        <v>-1.5875E-2</v>
-      </c>
-      <c r="I5">
+      <c r="G5" s="2">
+        <v>0.199045</v>
+      </c>
+      <c r="H5" s="2">
+        <v>-2.2771E-2</v>
+      </c>
+      <c r="I5" s="2">
+        <v>5.0075000000000001E-2</v>
+      </c>
+      <c r="J5" s="2">
+        <v>0.27860000000000001</v>
+      </c>
+      <c r="K5" s="2">
+        <v>1.7765E-2</v>
+      </c>
+      <c r="L5" s="2">
         <v>5.0201999999999997E-2</v>
       </c>
-      <c r="J5">
-        <v>0.27860000000000001</v>
-      </c>
-      <c r="K5">
-        <v>1.7765E-2</v>
-      </c>
-      <c r="L5">
-        <v>5.0201999999999997E-2</v>
-      </c>
-      <c r="M5">
-        <v>2</v>
-      </c>
-      <c r="N5">
-        <v>2</v>
-      </c>
-      <c r="O5">
+      <c r="M5" s="2">
+        <v>2</v>
+      </c>
+      <c r="N5" s="2">
+        <v>2</v>
+      </c>
+      <c r="O5" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P5">
+        <f t="shared" si="0"/>
+        <v>0.24731627942575879</v>
+      </c>
+      <c r="Q5">
+        <f t="shared" si="1"/>
+        <v>9.7368419209921235</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -722,44 +756,52 @@
       <c r="C6" t="s">
         <v>14</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="2">
         <v>-4.8259999999999997E-2</v>
       </c>
-      <c r="E6">
-        <v>2.1590000000000002E-2</v>
-      </c>
-      <c r="F6">
+      <c r="E6" s="2">
+        <v>2.0409E-2</v>
+      </c>
+      <c r="F6" s="2">
         <v>5.0075000000000001E-2</v>
       </c>
-      <c r="G6">
-        <v>0.26194499999999998</v>
-      </c>
-      <c r="H6">
-        <v>2.2225000000000002E-2</v>
-      </c>
-      <c r="I6">
+      <c r="G6" s="2">
+        <v>0.199045</v>
+      </c>
+      <c r="H6" s="2">
+        <v>2.0409E-2</v>
+      </c>
+      <c r="I6" s="2">
+        <v>5.0075000000000001E-2</v>
+      </c>
+      <c r="J6" s="2">
+        <v>0.275343</v>
+      </c>
+      <c r="K6" s="2">
+        <v>-1.7066000000000001E-2</v>
+      </c>
+      <c r="L6" s="2">
         <v>5.0201999999999997E-2</v>
       </c>
-      <c r="J6">
-        <v>0.275343</v>
-      </c>
-      <c r="K6">
-        <v>-1.7066000000000001E-2</v>
-      </c>
-      <c r="L6">
-        <v>5.0201999999999997E-2</v>
-      </c>
-      <c r="M6">
-        <v>2</v>
-      </c>
-      <c r="N6">
-        <v>2</v>
-      </c>
-      <c r="O6">
+      <c r="M6" s="2">
+        <v>2</v>
+      </c>
+      <c r="N6" s="2">
+        <v>2</v>
+      </c>
+      <c r="O6" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P6">
+        <f t="shared" si="0"/>
+        <v>0.247305</v>
+      </c>
+      <c r="Q6">
+        <f t="shared" si="1"/>
+        <v>9.7363978499999995</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>10</v>
       </c>
@@ -769,44 +811,52 @@
       <c r="C7" t="s">
         <v>14</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="2">
         <v>0.296205</v>
       </c>
-      <c r="E7">
-        <v>-1.7066000000000001E-2</v>
-      </c>
-      <c r="F7">
-        <v>5.0201999999999997E-2</v>
-      </c>
-      <c r="G7">
-        <v>0.50823399999999996</v>
-      </c>
-      <c r="H7">
-        <v>-1.1828E-2</v>
-      </c>
-      <c r="I7">
+      <c r="E7" s="2">
+        <v>-1.8246999999999999E-2</v>
+      </c>
+      <c r="F7" s="2">
+        <v>4.9439999999999998E-2</v>
+      </c>
+      <c r="G7" s="2">
+        <v>0.46731</v>
+      </c>
+      <c r="H7" s="2">
+        <v>-1.8246999999999999E-2</v>
+      </c>
+      <c r="I7" s="2">
+        <v>4.9439999999999998E-2</v>
+      </c>
+      <c r="J7" s="2">
+        <v>0.49303900000000001</v>
+      </c>
+      <c r="K7" s="2">
+        <v>2.0944999999999998E-2</v>
+      </c>
+      <c r="L7" s="2">
         <v>5.0265999999999998E-2</v>
       </c>
-      <c r="J7">
-        <v>0.49303900000000001</v>
-      </c>
-      <c r="K7">
-        <v>2.0944999999999998E-2</v>
-      </c>
-      <c r="L7">
-        <v>5.0265999999999998E-2</v>
-      </c>
-      <c r="M7">
+      <c r="M7" s="2">
         <v>3</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="2">
         <v>3</v>
       </c>
-      <c r="O7">
+      <c r="O7" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P7">
+        <f t="shared" si="0"/>
+        <v>0.17110500000000001</v>
+      </c>
+      <c r="Q7">
+        <f t="shared" si="1"/>
+        <v>6.7364038499999994</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -816,44 +866,52 @@
       <c r="C8" t="s">
         <v>14</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="2">
         <v>0.29591699999999999</v>
       </c>
-      <c r="E8">
-        <v>1.7066000000000001E-2</v>
-      </c>
-      <c r="F8">
-        <v>5.0201999999999997E-2</v>
-      </c>
-      <c r="G8">
-        <v>0.49911699999999998</v>
-      </c>
-      <c r="H8">
-        <v>1.5875E-2</v>
-      </c>
-      <c r="I8">
+      <c r="E8" s="2">
+        <v>1.5885E-2</v>
+      </c>
+      <c r="F8" s="2">
+        <v>4.9439999999999998E-2</v>
+      </c>
+      <c r="G8" s="2">
+        <v>0.46702199999999999</v>
+      </c>
+      <c r="H8" s="2">
+        <v>1.5885E-2</v>
+      </c>
+      <c r="I8" s="2">
+        <v>4.9439999999999998E-2</v>
+      </c>
+      <c r="J8" s="2">
+        <v>0.51663800000000004</v>
+      </c>
+      <c r="K8" s="2">
+        <v>1.2715000000000001E-2</v>
+      </c>
+      <c r="L8" s="2">
         <v>5.0265999999999998E-2</v>
       </c>
-      <c r="J8">
-        <v>0.51663800000000004</v>
-      </c>
-      <c r="K8">
-        <v>1.2715000000000001E-2</v>
-      </c>
-      <c r="L8">
-        <v>5.0265999999999998E-2</v>
-      </c>
-      <c r="M8">
+      <c r="M8" s="2">
         <v>3</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="2">
         <v>3</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P8">
+        <f t="shared" si="0"/>
+        <v>0.17110500000000001</v>
+      </c>
+      <c r="Q8">
+        <f t="shared" si="1"/>
+        <v>6.7364038499999994</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>3</v>
       </c>
@@ -863,44 +921,51 @@
       <c r="C9" t="s">
         <v>15</v>
       </c>
-      <c r="D9">
-        <v>-3.8563E-2</v>
-      </c>
-      <c r="E9">
-        <v>6.5709999999999996E-3</v>
-      </c>
-      <c r="F9">
-        <v>4.3947E-2</v>
-      </c>
-      <c r="G9">
-        <v>0.27233499999999999</v>
-      </c>
-      <c r="H9">
-        <v>-9.2189999999999998E-3</v>
-      </c>
-      <c r="I9">
+      <c r="D9" s="2">
+        <v>3.6311999999999997E-2</v>
+      </c>
+      <c r="E9" s="2">
+        <v>-6.3499999999999997E-3</v>
+      </c>
+      <c r="F9" s="2">
+        <v>3.8893999999999998E-2</v>
+      </c>
+      <c r="G9" s="2">
+        <v>0.26194499999999998</v>
+      </c>
+      <c r="H9" s="2">
+        <v>2.1044E-2</v>
+      </c>
+      <c r="I9" s="2">
+        <v>4.9947999999999999E-2</v>
+      </c>
+      <c r="J9" s="2">
+        <v>0.27860000000000001</v>
+      </c>
+      <c r="K9" s="2">
+        <v>1.7765E-2</v>
+      </c>
+      <c r="L9" s="2">
         <v>5.0158000000000001E-2</v>
       </c>
-      <c r="J9">
-        <v>0.27860000000000001</v>
-      </c>
-      <c r="K9">
-        <v>1.7765E-2</v>
-      </c>
-      <c r="L9">
-        <v>5.0158000000000001E-2</v>
-      </c>
-      <c r="M9">
+      <c r="M9" s="2">
         <v>0</v>
       </c>
-      <c r="N9">
-        <v>2</v>
-      </c>
-      <c r="O9">
+      <c r="N9" s="2">
+        <v>2</v>
+      </c>
+      <c r="O9" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P9">
+        <v>0.29175499999999999</v>
+      </c>
+      <c r="Q9">
+        <f t="shared" si="1"/>
+        <v>11.486394349999999</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -910,44 +975,51 @@
       <c r="C10" t="s">
         <v>15</v>
       </c>
-      <c r="D10">
-        <v>3.8563E-2</v>
-      </c>
-      <c r="E10">
-        <v>6.5709999999999996E-3</v>
-      </c>
-      <c r="F10">
-        <v>4.3947E-2</v>
-      </c>
-      <c r="G10">
+      <c r="D10" s="2">
+        <v>-3.8011000000000003E-2</v>
+      </c>
+      <c r="E10" s="2">
+        <v>-6.3499999999999997E-3</v>
+      </c>
+      <c r="F10" s="2">
+        <v>3.8893999999999998E-2</v>
+      </c>
+      <c r="G10" s="2">
         <v>0.26194499999999998</v>
       </c>
-      <c r="H10">
-        <v>2.2225000000000002E-2</v>
-      </c>
-      <c r="I10">
-        <v>5.0201999999999997E-2</v>
-      </c>
-      <c r="J10">
+      <c r="H10" s="2">
+        <v>-1.7056000000000002E-2</v>
+      </c>
+      <c r="I10" s="2">
+        <v>4.9947999999999999E-2</v>
+      </c>
+      <c r="J10" s="2">
         <v>0.275343</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="2">
         <v>-1.7066000000000001E-2</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="2">
         <v>4.7026999999999999E-2</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="2">
         <v>0</v>
       </c>
-      <c r="N10">
-        <v>2</v>
-      </c>
-      <c r="O10">
+      <c r="N10" s="2">
+        <v>2</v>
+      </c>
+      <c r="O10" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P10">
+        <v>0.29175499999999999</v>
+      </c>
+      <c r="Q10">
+        <f t="shared" si="1"/>
+        <v>11.486394349999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -957,129 +1029,153 @@
       <c r="C11" t="s">
         <v>15</v>
       </c>
-      <c r="D11">
-        <v>0.227965</v>
-      </c>
-      <c r="E11">
-        <v>0</v>
-      </c>
-      <c r="F11">
-        <v>5.0075500000000002E-2</v>
-      </c>
-      <c r="G11">
-        <v>0.49911699999999998</v>
-      </c>
-      <c r="H11">
-        <v>1.5875E-2</v>
-      </c>
-      <c r="I11">
+      <c r="D11" s="2">
+        <v>0.26229400000000003</v>
+      </c>
+      <c r="E11" s="2">
+        <v>-1.712E-3</v>
+      </c>
+      <c r="F11" s="2">
+        <v>2.6136E-2</v>
+      </c>
+      <c r="G11" s="2">
+        <v>0.46702199999999999</v>
+      </c>
+      <c r="H11" s="2">
+        <v>1.5885E-2</v>
+      </c>
+      <c r="I11" s="2">
+        <v>4.1598000000000003E-2</v>
+      </c>
+      <c r="J11" s="2">
+        <v>0.51663800000000004</v>
+      </c>
+      <c r="K11" s="2">
+        <v>1.2715000000000001E-2</v>
+      </c>
+      <c r="L11" s="2">
         <v>5.0265999999999998E-2</v>
       </c>
-      <c r="J11">
-        <v>0.51663800000000004</v>
-      </c>
-      <c r="K11">
-        <v>1.2715000000000001E-2</v>
-      </c>
-      <c r="L11">
-        <v>5.0265999999999998E-2</v>
-      </c>
-      <c r="M11">
-        <v>2</v>
-      </c>
-      <c r="N11">
+      <c r="M11" s="2">
+        <v>2</v>
+      </c>
+      <c r="N11" s="2">
         <v>4</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="P11">
+        <f t="shared" si="0"/>
+        <v>0.20490030490216452</v>
+      </c>
+      <c r="Q11">
+        <f t="shared" si="1"/>
+        <v>8.0669250039982163</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>31</v>
       </c>
       <c r="C12" t="s">
         <v>14</v>
       </c>
-      <c r="D12">
-        <v>3.5209999999999998E-2</v>
-      </c>
-      <c r="E12">
+      <c r="D12" s="2">
+        <v>3.3847000000000002E-2</v>
+      </c>
+      <c r="E12" s="2">
+        <v>-1.054E-3</v>
+      </c>
+      <c r="F12" s="2">
+        <v>7.76E-4</v>
+      </c>
+      <c r="G12" s="2">
+        <v>0.20340800000000001</v>
+      </c>
+      <c r="H12" s="2">
+        <v>-1.054E-3</v>
+      </c>
+      <c r="I12" s="2">
+        <v>2.3706000000000001E-2</v>
+      </c>
+      <c r="J12" s="2">
+        <v>0.24123</v>
+      </c>
+      <c r="K12" s="2">
         <v>0</v>
       </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <v>0.22434999999999999</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12">
+      <c r="L12" s="2">
         <v>3.4009999999999999E-2</v>
       </c>
-      <c r="J12">
-        <v>0.24123</v>
-      </c>
-      <c r="K12">
-        <v>0</v>
-      </c>
-      <c r="L12">
-        <v>3.4009999999999999E-2</v>
-      </c>
-      <c r="M12">
+      <c r="M12" s="2">
         <v>1</v>
       </c>
-      <c r="N12">
-        <v>2</v>
-      </c>
-      <c r="O12">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="N12" s="2">
+        <v>2</v>
+      </c>
+      <c r="O12" s="2">
+        <v>2</v>
+      </c>
+      <c r="P12">
+        <f t="shared" si="0"/>
+        <v>0.16800341609919725</v>
+      </c>
+      <c r="Q12">
+        <f t="shared" si="1"/>
+        <v>6.6142944918253956</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>32</v>
       </c>
       <c r="C13" t="s">
         <v>14</v>
       </c>
-      <c r="D13">
-        <v>3.5209999999999998E-2</v>
-      </c>
-      <c r="E13">
+      <c r="D13" s="2">
+        <v>3.3847000000000002E-2</v>
+      </c>
+      <c r="E13" s="2">
+        <v>-1.054E-3</v>
+      </c>
+      <c r="F13" s="2">
+        <v>9.9374000000000004E-2</v>
+      </c>
+      <c r="G13" s="2">
+        <v>0.20347100000000001</v>
+      </c>
+      <c r="H13" s="2">
+        <v>-1.054E-3</v>
+      </c>
+      <c r="I13" s="2">
+        <v>7.6911999999999994E-2</v>
+      </c>
+      <c r="J13" s="2">
+        <v>0.24123</v>
+      </c>
+      <c r="K13" s="2">
         <v>0</v>
       </c>
-      <c r="F13">
-        <v>9.6509999999999999E-2</v>
-      </c>
-      <c r="G13">
-        <v>0.22434999999999999</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
+      <c r="L13" s="2">
         <v>6.6390000000000005E-2</v>
       </c>
-      <c r="J13">
-        <v>0.24123</v>
-      </c>
-      <c r="K13">
-        <v>0</v>
-      </c>
-      <c r="L13">
-        <v>6.6390000000000005E-2</v>
-      </c>
-      <c r="M13">
+      <c r="M13" s="2">
         <v>1</v>
       </c>
-      <c r="N13">
-        <v>2</v>
-      </c>
-      <c r="O13">
-        <v>2</v>
+      <c r="N13" s="2">
+        <v>2</v>
+      </c>
+      <c r="O13" s="2">
+        <v>2</v>
+      </c>
+      <c r="P13">
+        <f t="shared" si="0"/>
+        <v>0.16813018745008285</v>
+      </c>
+      <c r="Q13">
+        <f t="shared" si="1"/>
+        <v>6.6192854799097613</v>
       </c>
     </row>
   </sheetData>

</xml_diff>